<commit_message>
Literature fixes, A1 outlier sensitivity check, status update
- Literature_Matrix.xlsx: correct metadata for [20], [22]-[24]; add [25]-[29]
  (AutoLiquid, LayoutPilot, AutoCompactionAI, Chettaoui & Hkiri, LST-Bench),
  DOIs verified on Crossref
- src/robustness_check.py: drop-the-outlier sensitivity check for noisy A1 cells
- Master document: status for Phases 6-7, literature section, Appendix A
- research_log: F-A1-6 (optimum plateau), decision to keep noisy cells
- docs/project_checklist.csv; openpyxl added to requirements-dev

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/literature/Literature_Matrix.xlsx
+++ b/literature/Literature_Matrix.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Literature Matrix" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Literature Matrix" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Notes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1641,12 +1641,12 @@
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>(various), arXiv</t>
+          <t>I. Chang</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>arXiv preprint, 2026</t>
+          <t>arXiv preprint 2603.02253, 2026 (not peer-reviewed)</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
@@ -1751,12 +1751,12 @@
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Yadwadkar et al.</t>
+          <t>Hsu, Nair, Menzies, Freeh</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>IEEE ICDCS, 2018</t>
+          <t>IEEE CLOUD, 2018</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
@@ -1801,12 +1801,12 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>Selecting the Best VM across Multiple Public Clouds (PARIS)</t>
+          <t>Selecting the Best VM across Multiple Public Clouds: A Data-Driven Performance Modeling Approach (PARIS)</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>Ortiz, Almanza, et al.</t>
+          <t>Yadwadkar, Hariharan, Gonzalez, Smith, Katz</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
@@ -1861,12 +1861,12 @@
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>(various)</t>
+          <t>Das Mohapatra, Oh</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>arXiv preprint, 2023</t>
+          <t>ACM/IFIP Middleware, 2023</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
@@ -1897,6 +1897,281 @@
       <c r="K25" s="7" t="inlineStr">
         <is>
           <t>Optimizes serverless-vs-VM resource choice; complementary to, but distinct from, your compaction/shuffle-tuning decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Table/data-layout optimization</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>AutoLiquid: Autonomic Data Layout Optimization for the Databricks Lakehouse</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>Nakandala, Bhanoori, Zhang, Negi, Sharma, et al. (Databricks)</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>PVLDB vol. 19, 2026</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>Choosing and maintaining clustering keys (vs. manual partitioning/Z-order) by hand does not keep up with evolving workloads</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>Autonomic system that proposes clustering-key changes from workload telemetry and verifies benefit before committing</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>Production Databricks lakehouse tables</t>
+        </is>
+      </c>
+      <c r="I26" s="7" t="inlineStr">
+        <is>
+          <t>Implicitly (verify-before-commit avoids unprofitable re-layouts)</t>
+        </is>
+      </c>
+      <c r="J26" s="7" t="inlineStr">
+        <is>
+          <t>Yes (core mechanism)</t>
+        </is>
+      </c>
+      <c r="K26" s="7" t="inlineStr">
+        <is>
+          <t>Industrial, telemetry-driven layout automation; no explicit break-even over future executions and not a dual-action (execution + storage) comparison</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Table/data-layout optimization</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>LayoutPilot: A Lakehouse Physical Design Advisor</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>Liu, Kipf, Borovica-Gajic</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>PVLDB vol. 19 (demo), 2026</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>Users lack evidence for choosing partitioning and intra-file layout (Z-order, clustering) at ingestion time</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>Interactive, workload-aware advisor that compares candidate layouts side by side on real workload evidence</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>Lakehouse workloads (demonstration)</t>
+        </is>
+      </c>
+      <c r="I27" s="7" t="inlineStr">
+        <is>
+          <t>Implicitly (benefit evidence before committing)</t>
+        </is>
+      </c>
+      <c r="J27" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K27" s="7" t="inlineStr">
+        <is>
+          <t>Advisory/what-if tooling for layout choice; leaves the 'is it worth it given N future runs' decision to the user - the question CAO-DF formalizes</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Data compaction</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>AutoCompactionAI: A Reinforcement Learning Framework for Adaptive File Compaction in Serverless Data Lakes</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>Venkatesan</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>IEEE FMLDS, 2025</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>When and how to compact small files in serverless data lakes (per title)</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>Reinforcement-learning framework for adaptive compaction (per title)</t>
+        </is>
+      </c>
+      <c r="H28" s="7" t="inlineStr">
+        <is>
+          <t>Serverless data lakes (per title)</t>
+        </is>
+      </c>
+      <c r="I28" s="7" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
+      <c r="J28" s="7" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
+      <c r="K28" s="7" t="inlineStr">
+        <is>
+          <t>Learned, opaque compaction policy vs. CAO-DF's interpretable break-even rule; also covers compaction only. [Metadata verified via Crossref; abstract not yet read - confirm before citing beyond title level.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Data compaction</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Correlation Aware Solution for Merging Small Files Based on Similarity and Clustering in HDFS</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Chettaoui, Hkiri</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>J. Supercomputing 81(15), Art. 1458, 2025</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>Small-file overhead in HDFS (per title)</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>Groups correlated/similar small files by clustering before merging (per title)</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>HDFS (per title)</t>
+        </is>
+      </c>
+      <c r="I29" s="7" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
+      <c r="J29" s="7" t="inlineStr">
+        <is>
+          <t>Partially (file correlation)</t>
+        </is>
+      </c>
+      <c r="K29" s="7" t="inlineStr">
+        <is>
+          <t>Optimizes *how* to merge small files; does not decide *whether* merging pays off over N runs. [Metadata verified via Crossref; abstract not yet read - confirm before citing beyond title level.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Data compaction</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>LST-Bench: Benchmarking Log-Structured Tables in the Cloud</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>Camacho-Rodriguez, Agrawal, Gruenheid, Gosalia, Petculescu, et al. (Microsoft)</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>Proc. ACM Manag. Data (SIGMOD) 2(1), 2024</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>Standard benchmarks miss the maintenance behaviour (compaction, mutations) of Delta/Iceberg/Hudi tables</t>
+        </is>
+      </c>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>Benchmark framework with longitudinal workloads including table maintenance operations</t>
+        </is>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>TPC-DS-based workloads on Delta Lake, Iceberg, Hudi</t>
+        </is>
+      </c>
+      <c r="I30" s="7" t="inlineStr">
+        <is>
+          <t>Partially (performance over time)</t>
+        </is>
+      </c>
+      <c r="J30" s="7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K30" s="7" t="inlineStr">
+        <is>
+          <t>Benchmarks how LST performance evolves over time and under maintenance (incl. compaction); measures effects but provides no decision rule for when maintenance pays off. (2024, slightly older than the 2025-26 target.)</t>
         </is>
       </c>
     </row>
@@ -1994,7 +2269,7 @@
         </is>
       </c>
       <c r="C4" s="9" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
@@ -2014,7 +2289,7 @@
         </is>
       </c>
       <c r="C5" s="9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>

</xml_diff>